<commit_message>
Agrega diagramas ERD y consultas de referencia (FIC-351 y Info_Portafolio)
</commit_message>
<xml_diff>
--- a/Documentación_bases_SIF.xlsx
+++ b/Documentación_bases_SIF.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://patriainvest-my.sharepoint.com/personal/emmanuel_palma_patria_com/Documents/Producción/Utilidades/Colombia/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{64119DAA-00BC-4B27-927D-984AD6798427}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EB615938-72B2-44FC-8563-B6EE17B94BD5}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{64119DAA-00BC-4B27-927D-984AD6798427}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F28E2974-E412-43CF-9DA7-B3D8161D5534}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{0D62D5E2-9F97-48A8-B65A-54DD2A8B7EE0}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{0D62D5E2-9F97-48A8-B65A-54DD2A8B7EE0}"/>
   </bookViews>
   <sheets>
     <sheet name="Parámetros" sheetId="4" state="hidden" r:id="rId1"/>
@@ -3050,8 +3050,8 @@
     <col min="2" max="2" width="30" style="3" customWidth="1"/>
     <col min="3" max="3" width="47" style="3" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="45.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="38.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="83.5703125" style="3" customWidth="1"/>
+    <col min="5" max="5" width="38.42578125" style="3" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="83.5703125" style="3" hidden="1" customWidth="1"/>
     <col min="7" max="7" width="12.140625" style="3" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="25.28515625" style="3" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="27.5703125" bestFit="1" customWidth="1"/>

</xml_diff>